<commit_message>
Revision 1 for Ecology_MQ
</commit_message>
<xml_diff>
--- a/Data/Pond plant transplanting result-2019/DI.xlsx
+++ b/Data/Pond plant transplanting result-2019/DI.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10609"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{995EA1FD-C164-124A-B1F3-464DD23EC344}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97CD7BF9-8915-CE48-ACAD-3A691AAABF48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="640" windowWidth="30240" windowHeight="17980" tabRatio="863" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="640" windowWidth="30240" windowHeight="17980" tabRatio="863" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plant growth" sheetId="1" r:id="rId1"/>
@@ -13,6 +13,7 @@
     <sheet name="Biomass" sheetId="9" r:id="rId3"/>
     <sheet name="Flowering" sheetId="10" r:id="rId4"/>
     <sheet name="Salinity" sheetId="6" r:id="rId5"/>
+    <sheet name="Survival rate" sheetId="11" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Biomass!$B$1:$B$56</definedName>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3346" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3404" uniqueCount="150">
   <si>
     <t>ID</t>
   </si>
@@ -523,6 +524,15 @@
   <si>
     <t>Neighbor removal</t>
   </si>
+  <si>
+    <t>Site</t>
+  </si>
+  <si>
+    <t>Survival rate (%)</t>
+  </si>
+  <si>
+    <t>Deal Island</t>
+  </si>
 </sst>
 </file>
 
@@ -531,7 +541,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]mmm\-yy;@"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -601,6 +611,12 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="6">
@@ -23862,4 +23878,285 @@
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2BAD1E68-FDA3-564F-8599-A040E96DB051}">
+  <dimension ref="A1:D19"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="16.33203125" customWidth="1"/>
+    <col min="4" max="4" width="10.83203125" style="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" t="s">
+        <v>147</v>
+      </c>
+      <c r="B1" t="s">
+        <v>142</v>
+      </c>
+      <c r="C1" t="s">
+        <v>148</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
+        <v>149</v>
+      </c>
+      <c r="B2" t="s">
+        <v>141</v>
+      </c>
+      <c r="C2">
+        <v>100</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" t="s">
+        <v>149</v>
+      </c>
+      <c r="B3" t="s">
+        <v>140</v>
+      </c>
+      <c r="C3">
+        <v>100</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" t="s">
+        <v>149</v>
+      </c>
+      <c r="B4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C4">
+        <v>100</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" t="s">
+        <v>149</v>
+      </c>
+      <c r="B5" t="s">
+        <v>145</v>
+      </c>
+      <c r="C5">
+        <v>100</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" t="s">
+        <v>149</v>
+      </c>
+      <c r="B6" t="s">
+        <v>146</v>
+      </c>
+      <c r="C6">
+        <v>100</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" t="s">
+        <v>149</v>
+      </c>
+      <c r="B7" t="s">
+        <v>70</v>
+      </c>
+      <c r="C7">
+        <v>100</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" t="s">
+        <v>149</v>
+      </c>
+      <c r="B8" t="s">
+        <v>141</v>
+      </c>
+      <c r="C8">
+        <v>80</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" t="s">
+        <v>149</v>
+      </c>
+      <c r="B9" t="s">
+        <v>140</v>
+      </c>
+      <c r="C9">
+        <v>100</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" t="s">
+        <v>149</v>
+      </c>
+      <c r="B10" t="s">
+        <v>61</v>
+      </c>
+      <c r="C10">
+        <v>100</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" t="s">
+        <v>149</v>
+      </c>
+      <c r="B11" t="s">
+        <v>145</v>
+      </c>
+      <c r="C11">
+        <v>100</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" t="s">
+        <v>149</v>
+      </c>
+      <c r="B12" t="s">
+        <v>146</v>
+      </c>
+      <c r="C12">
+        <v>100</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13" t="s">
+        <v>149</v>
+      </c>
+      <c r="B13" t="s">
+        <v>70</v>
+      </c>
+      <c r="C13">
+        <v>100</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" t="s">
+        <v>149</v>
+      </c>
+      <c r="B14" t="s">
+        <v>141</v>
+      </c>
+      <c r="C14">
+        <v>10</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="A15" t="s">
+        <v>149</v>
+      </c>
+      <c r="B15" t="s">
+        <v>140</v>
+      </c>
+      <c r="C15">
+        <v>100</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="A16" t="s">
+        <v>149</v>
+      </c>
+      <c r="B16" t="s">
+        <v>61</v>
+      </c>
+      <c r="C16">
+        <v>100</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
+      <c r="A17" t="s">
+        <v>149</v>
+      </c>
+      <c r="B17" t="s">
+        <v>145</v>
+      </c>
+      <c r="C17">
+        <v>100</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
+      <c r="A18" t="s">
+        <v>149</v>
+      </c>
+      <c r="B18" t="s">
+        <v>146</v>
+      </c>
+      <c r="C18">
+        <v>100</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
+      <c r="A19" t="s">
+        <v>149</v>
+      </c>
+      <c r="B19" t="s">
+        <v>70</v>
+      </c>
+      <c r="C19">
+        <v>100</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>119</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="11" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>